<commit_message>
Update ESP32 PCB projects and generated assets
</commit_message>
<xml_diff>
--- a/ESP32_S3_MINI_1/BOM.xlsx
+++ b/ESP32_S3_MINI_1/BOM.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="BOM" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="BOM" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -424,16 +424,16 @@
     <t xml:space="preserve">BOOMELE</t>
   </si>
   <si>
-    <t xml:space="preserve">1.0T-4P</t>
+    <t xml:space="preserve">1.0T-4PLTPZ</t>
   </si>
   <si>
     <t xml:space="preserve">Qwiic_Vertical</t>
   </si>
   <si>
-    <t xml:space="preserve">C970137</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.lcsc.com/product-detail/C970137.html?s_z=n_C970137</t>
+    <t xml:space="preserve">C2974722</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcsc.com/product-detail/C2974722.html</t>
   </si>
   <si>
     <t xml:space="preserve">J7,J4</t>
@@ -779,7 +779,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -823,22 +823,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <u val="single"/>
-      <sz val="10"/>
-      <color rgb="FF0563C1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <u val="single"/>
-      <sz val="11"/>
-      <color rgb="FF0563C1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -860,7 +844,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -868,8 +852,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -893,64 +884,64 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -976,7 +967,7 @@
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0563C1"/>
+      <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFCCCCFF"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -1015,1612 +1006,1719 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q38"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="33.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="14.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="23.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="23.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="14.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="7.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.86"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="23.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="14.21"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="K2" s="5" t="n">
         <v>0.32</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="L2" s="5" t="n">
         <f aca="false">K2*D2</f>
         <v>1.6</v>
       </c>
-      <c r="P2" s="4"/>
+      <c r="P2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <f aca="false">A2+1</f>
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="K3" s="5" t="n">
         <v>0.13</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="L3" s="5" t="n">
         <f aca="false">K3*D3</f>
         <v>0.13</v>
       </c>
-      <c r="P3" s="4"/>
+      <c r="P3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <f aca="false">A3+1</f>
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="J4" s="5" t="s">
+      <c r="J4" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="5" t="n">
         <v>0.57</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="5" t="n">
         <f aca="false">K4*D4</f>
         <v>0.57</v>
       </c>
-      <c r="P4" s="4"/>
+      <c r="P4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <f aca="false">A4+1</f>
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K5" s="5" t="n">
         <v>0.58</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="L5" s="5" t="n">
         <f aca="false">K5*D5</f>
         <v>2.32</v>
       </c>
-      <c r="P5" s="4"/>
+      <c r="P5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <f aca="false">A5+1</f>
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="K6" s="5" t="n">
         <v>0.96</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="L6" s="5" t="n">
         <f aca="false">K6*D6</f>
         <v>1.92</v>
       </c>
-      <c r="P6" s="4"/>
+      <c r="P6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <f aca="false">A6+1</f>
         <v>6</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="0" t="s">
+      <c r="G7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="K7" s="5" t="n">
         <v>0.81</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="L7" s="5" t="n">
         <f aca="false">K7*D7</f>
         <v>0.81</v>
       </c>
-      <c r="P7" s="4"/>
+      <c r="P7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="5" t="n">
         <f aca="false">A7+1</f>
         <v>7</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D8" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="K8" s="5" t="n">
         <v>0.04</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="L8" s="5" t="n">
         <f aca="false">K8*D8</f>
         <v>0.04</v>
       </c>
-      <c r="M8" s="0" t="s">
+      <c r="M8" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="N8" s="0" t="s">
+      <c r="N8" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="O8" s="0" t="n">
+      <c r="O8" s="1" t="n">
         <v>0.1</v>
       </c>
-      <c r="P8" s="4"/>
+      <c r="P8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="5" t="n">
         <f aca="false">A8+1</f>
         <v>8</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D9" s="0" t="n">
+      <c r="D9" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="K9" s="4" t="n">
+      <c r="K9" s="5" t="n">
         <v>0.19</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="L9" s="5" t="n">
         <f aca="false">K9*D9</f>
         <v>0.19</v>
       </c>
-      <c r="M9" s="0" t="s">
+      <c r="M9" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="N9" s="0" t="s">
+      <c r="N9" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="O9" s="0" t="n">
+      <c r="O9" s="1" t="n">
         <v>0.34</v>
       </c>
-      <c r="P9" s="4"/>
+      <c r="P9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="5" t="n">
         <f aca="false">A9+1</f>
         <v>9</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="0" t="n">
+      <c r="D10" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="G10" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="J10" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="K10" s="4" t="n">
+      <c r="K10" s="5" t="n">
         <v>0.17</v>
       </c>
-      <c r="L10" s="4" t="n">
+      <c r="L10" s="5" t="n">
         <f aca="false">K10*D10</f>
         <v>0.17</v>
       </c>
-      <c r="M10" s="0" t="s">
+      <c r="M10" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="N10" s="0" t="s">
+      <c r="N10" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="O10" s="0" t="n">
+      <c r="O10" s="1" t="n">
         <v>0.24</v>
       </c>
-      <c r="P10" s="4"/>
+      <c r="P10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="5" t="n">
         <f aca="false">A10+1</f>
         <v>10</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="0" t="n">
+      <c r="D11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="G11" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="J11" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="K11" s="4" t="n">
+      <c r="K11" s="5" t="n">
         <v>0.2</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="L11" s="5" t="n">
         <f aca="false">K11*D11</f>
         <v>0.4</v>
       </c>
-      <c r="M11" s="0" t="s">
+      <c r="M11" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="N11" s="0" t="s">
+      <c r="N11" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="O11" s="0" t="n">
+      <c r="O11" s="1" t="n">
         <v>0.27</v>
       </c>
-      <c r="P11" s="4"/>
+      <c r="P11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="5" t="n">
         <f aca="false">A11+1</f>
         <v>11</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D12" s="0" t="n">
+      <c r="D12" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="G12" s="0" t="s">
+      <c r="G12" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="J12" s="5" t="s">
+      <c r="J12" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="K12" s="4" t="n">
+      <c r="K12" s="5" t="n">
         <v>0.45</v>
       </c>
-      <c r="L12" s="4" t="n">
+      <c r="L12" s="5" t="n">
         <f aca="false">K12*D12</f>
         <v>0.45</v>
       </c>
-      <c r="P12" s="4"/>
+      <c r="P12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="5" t="n">
         <f aca="false">A12+1</f>
         <v>12</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="F13" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G13" s="0" t="s">
+      <c r="G13" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="K13" s="6" t="n">
+      <c r="K13" s="7" t="n">
         <v>0.56</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="L13" s="5" t="n">
         <f aca="false">K13*D13</f>
         <v>1.12</v>
       </c>
-      <c r="M13" s="0" t="s">
+      <c r="M13" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="N13" s="0" t="s">
+      <c r="N13" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="O13" s="0" t="n">
+      <c r="O13" s="1" t="n">
         <v>0.26</v>
       </c>
-      <c r="P13" s="4"/>
+      <c r="P13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="5" t="n">
         <f aca="false">A13+1</f>
         <v>13</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D14" s="0" t="n">
+      <c r="D14" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="F14" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="K14" s="4" t="n">
+      <c r="K14" s="5" t="n">
         <v>1.17</v>
       </c>
-      <c r="L14" s="4" t="n">
+      <c r="L14" s="5" t="n">
         <f aca="false">K14*D14</f>
         <v>1.17</v>
       </c>
-      <c r="M14" s="0" t="s">
+      <c r="M14" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="N14" s="0" t="s">
+      <c r="N14" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="O14" s="0" t="n">
+      <c r="O14" s="1" t="n">
         <v>1.25</v>
       </c>
-      <c r="P14" s="4"/>
+      <c r="P14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="5" t="n">
         <f aca="false">A14+1</f>
         <v>14</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="D15" s="0" t="n">
+      <c r="D15" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="F15" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G15" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="H15" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J15" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="K15" s="4" t="n">
+      <c r="K15" s="5" t="n">
         <v>1.9</v>
       </c>
-      <c r="L15" s="4" t="n">
+      <c r="L15" s="5" t="n">
         <f aca="false">K15*D15</f>
         <v>1.9</v>
       </c>
-      <c r="M15" s="0" t="s">
+      <c r="M15" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="N15" s="0" t="s">
+      <c r="N15" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="O15" s="0" t="n">
+      <c r="O15" s="1" t="n">
         <v>2.03</v>
       </c>
-      <c r="P15" s="4"/>
+      <c r="P15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="n">
+      <c r="A16" s="5" t="n">
         <f aca="false">A15+1</f>
         <v>15</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="D16" s="0" t="n">
+      <c r="D16" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="F16" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="G16" s="0" t="s">
+      <c r="G16" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="H16" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="J16" s="5" t="s">
+      <c r="J16" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="K16" s="4" t="n">
+      <c r="K16" s="5" t="n">
         <v>0.2</v>
       </c>
-      <c r="L16" s="4" t="n">
+      <c r="L16" s="5" t="n">
         <f aca="false">K16*D16</f>
         <v>0.2</v>
       </c>
-      <c r="M16" s="0" t="s">
+      <c r="M16" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="N16" s="0" t="s">
+      <c r="N16" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="O16" s="0" t="n">
+      <c r="O16" s="1" t="n">
         <v>0.49</v>
       </c>
-      <c r="P16" s="4"/>
+      <c r="P16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="5" t="n">
         <f aca="false">A16+1</f>
         <v>16</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="D17" s="0" t="n">
+      <c r="D17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="F17" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="G17" s="0" t="s">
+      <c r="G17" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="H17" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="I17" s="4" t="s">
+      <c r="I17" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="J17" s="5" t="s">
+      <c r="J17" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="K17" s="6" t="n">
+      <c r="K17" s="7" t="n">
         <v>1.31</v>
       </c>
-      <c r="L17" s="4" t="n">
+      <c r="L17" s="5" t="n">
         <f aca="false">K17*D17</f>
         <v>1.31</v>
       </c>
-      <c r="M17" s="0" t="s">
+      <c r="M17" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="N17" s="0" t="s">
+      <c r="N17" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="O17" s="0" t="n">
+      <c r="O17" s="1" t="n">
         <v>0.86</v>
       </c>
-      <c r="P17" s="4"/>
+      <c r="P17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="5" t="n">
         <f aca="false">A17+1</f>
         <v>17</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="D18" s="0" t="n">
+      <c r="D18" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="F18" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="H18" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="I18" s="0" t="s">
+      <c r="I18" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="J18" s="7" t="s">
+      <c r="J18" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="K18" s="4" t="n">
+      <c r="K18" s="5" t="n">
         <v>0.65</v>
       </c>
-      <c r="L18" s="4" t="n">
+      <c r="L18" s="5" t="n">
         <f aca="false">K18*D18</f>
         <v>0.65</v>
       </c>
-      <c r="P18" s="4"/>
+      <c r="P18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="5" t="n">
         <f aca="false">A18+1</f>
         <v>18</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="D19" s="0" t="n">
+      <c r="D19" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F19" s="0" t="s">
+      <c r="F19" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="H19" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4" t="s">
+      <c r="I19" s="5"/>
+      <c r="J19" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="P19" s="4"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="P19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="5" t="n">
         <f aca="false">A19+1</f>
         <v>19</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D20" s="0" t="n">
+      <c r="D20" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="H20" s="0" t="s">
+      <c r="H20" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4" t="s">
+      <c r="I20" s="5"/>
+      <c r="J20" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="P20" s="4"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="P20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="5" t="n">
         <f aca="false">A20+1</f>
         <v>20</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D21" s="0" t="n">
+      <c r="D21" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="E21" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="H21" s="0" t="s">
+      <c r="H21" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4" t="s">
+      <c r="I21" s="5"/>
+      <c r="J21" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="P21" s="4"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="P21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="5" t="n">
         <f aca="false">A21+1</f>
         <v>21</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D22" s="0" t="n">
+      <c r="D22" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="0" t="s">
+      <c r="E22" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F22" s="0" t="s">
+      <c r="F22" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="H22" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="I22" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="J22" s="5" t="s">
+      <c r="J22" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="K22" s="4" t="n">
+      <c r="K22" s="5" t="n">
         <v>0.13</v>
       </c>
-      <c r="L22" s="4" t="n">
+      <c r="L22" s="5" t="n">
         <f aca="false">K22*D22</f>
         <v>0.13</v>
       </c>
-      <c r="M22" s="0" t="s">
+      <c r="M22" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="N22" s="0" t="s">
+      <c r="N22" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="O22" s="0" t="n">
+      <c r="O22" s="1" t="n">
         <v>0.25</v>
       </c>
-      <c r="P22" s="4"/>
+      <c r="P22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="5" t="n">
         <f aca="false">A22+1</f>
         <v>22</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D23" s="0" t="n">
+      <c r="D23" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G23" s="0" t="s">
+      <c r="G23" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="H23" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="I23" s="4" t="s">
+      <c r="I23" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="J23" s="5" t="s">
+      <c r="J23" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="K23" s="4" t="n">
+      <c r="K23" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="L23" s="4" t="n">
+      <c r="L23" s="5" t="n">
         <f aca="false">K23*D23</f>
         <v>0.16</v>
       </c>
-      <c r="P23" s="4"/>
+      <c r="P23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="5" t="n">
         <f aca="false">A23+1</f>
         <v>23</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D24" s="0" t="n">
+      <c r="D24" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G24" s="0" t="s">
+      <c r="G24" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="H24" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="J24" s="5" t="s">
+      <c r="J24" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="K24" s="4" t="n">
+      <c r="K24" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="L24" s="4" t="n">
+      <c r="L24" s="5" t="n">
         <f aca="false">K24*D24</f>
         <v>0.16</v>
       </c>
-      <c r="P24" s="4"/>
+      <c r="P24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="5" t="n">
         <f aca="false">A24+1</f>
         <v>24</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="C25" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D25" s="0" t="n">
+      <c r="D25" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G25" s="0" t="s">
+      <c r="G25" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="H25" s="1" t="n">
+      <c r="H25" s="2" t="n">
         <v>330</v>
       </c>
-      <c r="I25" s="4" t="s">
+      <c r="I25" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="J25" s="5" t="s">
+      <c r="J25" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="K25" s="4" t="n">
+      <c r="K25" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="L25" s="4" t="n">
+      <c r="L25" s="5" t="n">
         <f aca="false">K25*D25</f>
         <v>0.08</v>
       </c>
-      <c r="P25" s="4"/>
+      <c r="P25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="5" t="n">
         <f aca="false">A25+1</f>
         <v>25</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D26" s="0" t="n">
+      <c r="D26" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="0" t="s">
+      <c r="G26" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="H26" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="I26" s="4" t="s">
+      <c r="I26" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="J26" s="5" t="s">
+      <c r="J26" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="K26" s="4" t="n">
+      <c r="K26" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="L26" s="4" t="n">
+      <c r="L26" s="5" t="n">
         <f aca="false">K26*D26</f>
         <v>0.08</v>
       </c>
-      <c r="P26" s="4"/>
+      <c r="P26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="5" t="n">
         <f aca="false">A26+1</f>
         <v>26</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="C27" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D27" s="0" t="n">
+      <c r="D27" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G27" s="0" t="s">
+      <c r="G27" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="H27" s="1" t="n">
+      <c r="H27" s="2" t="n">
         <v>300</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="I27" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="J27" s="5" t="s">
+      <c r="J27" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="K27" s="4" t="n">
+      <c r="K27" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="L27" s="4" t="n">
+      <c r="L27" s="5" t="n">
         <f aca="false">K27*D27</f>
         <v>0.08</v>
       </c>
-      <c r="P27" s="4"/>
+      <c r="P27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="5" t="n">
         <f aca="false">A27+1</f>
         <v>27</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C28" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D28" s="0" t="n">
+      <c r="D28" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G28" s="0" t="s">
+      <c r="G28" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="H28" s="1" t="s">
+      <c r="H28" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="I28" s="4" t="s">
+      <c r="I28" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="J28" s="5" t="s">
+      <c r="J28" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="K28" s="4" t="n">
+      <c r="K28" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="L28" s="4" t="n">
+      <c r="L28" s="5" t="n">
         <f aca="false">K28*D28</f>
         <v>0.16</v>
       </c>
-      <c r="P28" s="4"/>
+      <c r="P28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="5" t="n">
         <f aca="false">A28+1</f>
         <v>28</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="C29" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D29" s="0" t="n">
+      <c r="D29" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E29" s="4" t="s">
+      <c r="E29" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G29" s="0" t="s">
+      <c r="G29" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="H29" s="1" t="s">
+      <c r="H29" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="I29" s="4" t="s">
+      <c r="I29" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="J29" s="5" t="s">
+      <c r="J29" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="K29" s="4" t="n">
+      <c r="K29" s="5" t="n">
         <v>0.09</v>
       </c>
-      <c r="L29" s="4" t="n">
+      <c r="L29" s="5" t="n">
         <f aca="false">K29*D29</f>
         <v>0.36</v>
       </c>
-      <c r="P29" s="4"/>
+      <c r="P29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="5" t="n">
         <f aca="false">A29+1</f>
         <v>29</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="C30" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="D30" s="0" t="n">
+      <c r="D30" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E30" s="0" t="s">
+      <c r="E30" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="G30" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="H30" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="I30" s="4" t="s">
+      <c r="I30" s="5" t="s">
         <v>197</v>
       </c>
-      <c r="J30" s="5" t="s">
+      <c r="J30" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="K30" s="6" t="n">
+      <c r="K30" s="7" t="n">
         <v>1.72</v>
       </c>
-      <c r="L30" s="4" t="n">
+      <c r="L30" s="5" t="n">
         <f aca="false">K30*D30</f>
         <v>3.44</v>
       </c>
-      <c r="M30" s="0" t="s">
+      <c r="M30" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="N30" s="0" t="s">
+      <c r="N30" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="O30" s="0" t="n">
+      <c r="O30" s="1" t="n">
         <v>0.4</v>
       </c>
-      <c r="P30" s="4"/>
+      <c r="P30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="5" t="n">
         <f aca="false">A30+1</f>
         <v>30</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="C31" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D31" s="0" t="n">
+      <c r="D31" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E31" s="0" t="s">
+      <c r="E31" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G31" s="0" t="s">
+      <c r="G31" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="H31" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="I31" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="J31" s="5" t="s">
+      <c r="J31" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="K31" s="4" t="n">
+      <c r="K31" s="5" t="n">
         <v>0.08</v>
       </c>
-      <c r="L31" s="4" t="n">
+      <c r="L31" s="5" t="n">
         <f aca="false">K31*D31</f>
         <v>0.16</v>
       </c>
-      <c r="P31" s="4"/>
+      <c r="P31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="5" t="n">
         <f aca="false">A31+1</f>
         <v>31</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="C32" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D32" s="0" t="n">
+      <c r="D32" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="0" t="s">
+      <c r="E32" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="F32" s="0" t="s">
+      <c r="F32" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="G32" s="0" t="s">
+      <c r="G32" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="H32" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="I32" s="4" t="s">
+      <c r="I32" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="J32" s="5" t="s">
+      <c r="J32" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="K32" s="4" t="n">
+      <c r="K32" s="5" t="n">
         <v>0.01</v>
       </c>
-      <c r="L32" s="4" t="n">
+      <c r="L32" s="5" t="n">
         <f aca="false">K32*D32</f>
         <v>0.01</v>
       </c>
-      <c r="P32" s="4"/>
+      <c r="P32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="5" t="n">
         <f aca="false">A32+1</f>
         <v>32</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="B33" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="C33" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="D33" s="0" t="n">
+      <c r="D33" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="0" t="s">
+      <c r="E33" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="F33" s="0" t="s">
+      <c r="F33" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="G33" s="8" t="s">
+      <c r="G33" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="H33" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="I33" s="8" t="s">
+      <c r="I33" s="9" t="s">
         <v>219</v>
       </c>
-      <c r="J33" s="9" t="s">
+      <c r="J33" s="10" t="s">
         <v>220</v>
       </c>
-      <c r="K33" s="8" t="n">
+      <c r="K33" s="9" t="n">
         <v>4.6185</v>
       </c>
-      <c r="L33" s="4" t="n">
+      <c r="L33" s="5" t="n">
         <f aca="false">K33*D33</f>
         <v>4.6185</v>
       </c>
-      <c r="P33" s="4"/>
+      <c r="P33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="n">
+      <c r="A34" s="5" t="n">
         <f aca="false">A33+1</f>
         <v>33</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="B34" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="C34" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="D34" s="0" t="n">
+      <c r="D34" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="0" t="s">
+      <c r="E34" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="F34" s="0" t="s">
+      <c r="F34" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="G34" s="0" t="s">
+      <c r="G34" s="1" t="s">
         <v>225</v>
       </c>
-      <c r="H34" s="1" t="s">
+      <c r="H34" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="I34" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="J34" s="5" t="s">
+      <c r="J34" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="K34" s="4" t="n">
+      <c r="K34" s="5" t="n">
         <v>2.66</v>
       </c>
-      <c r="L34" s="4" t="n">
+      <c r="L34" s="5" t="n">
         <f aca="false">K34*D34</f>
         <v>2.66</v>
       </c>
-      <c r="M34" s="0" t="s">
+      <c r="M34" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="N34" s="0" t="s">
+      <c r="N34" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="O34" s="0" t="n">
+      <c r="O34" s="1" t="n">
         <v>5.77</v>
       </c>
-      <c r="P34" s="4"/>
+      <c r="P34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="n">
+      <c r="A35" s="5" t="n">
         <f aca="false">A34+1</f>
         <v>34</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="C35" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="D35" s="0" t="n">
+      <c r="D35" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E35" s="0" t="s">
+      <c r="E35" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="F35" s="0" t="s">
+      <c r="F35" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="G35" s="0" t="s">
+      <c r="G35" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="H35" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="I35" s="4" t="s">
+      <c r="I35" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="J35" s="5" t="s">
+      <c r="J35" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="K35" s="4" t="n">
+      <c r="K35" s="5" t="n">
         <v>0.22</v>
       </c>
-      <c r="L35" s="4" t="n">
+      <c r="L35" s="5" t="n">
         <f aca="false">K35*D35</f>
         <v>0.22</v>
       </c>
-      <c r="M35" s="0" t="s">
+      <c r="M35" s="1" t="s">
         <v>239</v>
       </c>
-      <c r="N35" s="0" t="s">
+      <c r="N35" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="O35" s="0" t="n">
+      <c r="O35" s="1" t="n">
         <v>1.52</v>
       </c>
-      <c r="P35" s="4"/>
+      <c r="P35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="n">
+      <c r="A36" s="5" t="n">
         <f aca="false">A35+1</f>
         <v>35</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="B36" s="1" t="s">
         <v>241</v>
       </c>
-      <c r="C36" s="0" t="s">
+      <c r="C36" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="D36" s="0" t="n">
+      <c r="D36" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E36" s="0" t="s">
+      <c r="E36" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="F36" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="G36" s="0" t="s">
+      <c r="G36" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="H36" s="2" t="s">
         <v>245</v>
       </c>
-      <c r="I36" s="4" t="s">
+      <c r="I36" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="J36" s="5" t="s">
+      <c r="J36" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="K36" s="10" t="n">
+      <c r="K36" s="11" t="n">
         <v>0.88</v>
       </c>
-      <c r="L36" s="4" t="n">
+      <c r="L36" s="5" t="n">
         <f aca="false">K36*D36</f>
         <v>1.76</v>
       </c>
-      <c r="M36" s="0" t="s">
+      <c r="M36" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="N36" s="5" t="s">
+      <c r="N36" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="O36" s="0" t="n">
+      <c r="O36" s="1" t="n">
         <v>0.85</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="P37" s="4"/>
-      <c r="Q37" s="4"/>
+      <c r="P37" s="5"/>
+      <c r="Q37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L38" s="0" t="n">
+      <c r="L38" s="1" t="n">
         <f aca="false">SUM(L2:L36)</f>
         <v>29.0285</v>
       </c>
@@ -2643,23 +2741,22 @@
     <hyperlink ref="J15" r:id="rId14" display="https://www.lcsc.com/product-detail/C19725033.html?s_z=n_C19725033"/>
     <hyperlink ref="J16" r:id="rId15" display="https://www.lcsc.com/product-detail/C295747.html?s_z=n_C295747"/>
     <hyperlink ref="J17" r:id="rId16" display="https://www.lcsc.com/product-detail/C3445864.html?s_z=n_C3445864"/>
-    <hyperlink ref="J18" r:id="rId17" display="https://www.lcsc.com/product-detail/C970137.html?s_z=n_C970137"/>
-    <hyperlink ref="J22" r:id="rId18" display="https://www.lcsc.com/product-detail/C695609.html?s_z=n_C695609"/>
-    <hyperlink ref="J23" r:id="rId19" display="https://www.lcsc.com/product-detail/C60491.html?s_z=n_C60491"/>
-    <hyperlink ref="J24" r:id="rId20" display="https://www.lcsc.com/product-detail/C105871.html?s_z=n_C105871"/>
-    <hyperlink ref="J25" r:id="rId21" display="https://www.lcsc.com/product-detail/C105875.html?s_z=n_C105875"/>
-    <hyperlink ref="J26" r:id="rId22" display="https://www.lcsc.com/product-detail/C138044.html?s_z=n_C138044"/>
-    <hyperlink ref="J27" r:id="rId23" display="https://www.lcsc.com/product-detail/C138010.html?s_z=n_C138010"/>
-    <hyperlink ref="J28" r:id="rId24" display="https://www.lcsc.com/product-detail/C105872.html?s_z=n_C105872"/>
-    <hyperlink ref="J29" r:id="rId25" display="https://www.lcsc.com/product-detail/C114762.html?s_z=n_C114762"/>
-    <hyperlink ref="J30" r:id="rId26" display="https://www.lcsc.com/product-detail/C2760981.html?s_z=n_C2760981"/>
-    <hyperlink ref="J31" r:id="rId27" display="https://www.lcsc.com/product-detail/C60490.html?s_z=n_C60490"/>
-    <hyperlink ref="J32" r:id="rId28" display="https://www.lcsc.com/product-detail/C77131.html?s_z=n_C77131"/>
-    <hyperlink ref="J33" r:id="rId29" display="https://www.lcsc.com/product-detail/C2913206.html?s_z=n_C2913206"/>
-    <hyperlink ref="J34" r:id="rId30" display="https://www.lcsc.com/product-detail/C2682616.html?s_z=n_C2682616"/>
-    <hyperlink ref="J35" r:id="rId31" display="https://www.lcsc.com/product-detail/C99269.html?s_z=n_C99269"/>
-    <hyperlink ref="J36" r:id="rId32" display="https://www.lcsc.com/product-detail/C2869734.html?s_z=n_C2869734"/>
-    <hyperlink ref="N36" r:id="rId33" display="https://www.mouser.com/ProductDetail/Texas-Instruments/LM66100DCKT?qs=vLWxofP3U2zoiBCtDTudjw%3D%3D"/>
+    <hyperlink ref="J22" r:id="rId17" display="https://www.lcsc.com/product-detail/C695609.html?s_z=n_C695609"/>
+    <hyperlink ref="J23" r:id="rId18" display="https://www.lcsc.com/product-detail/C60491.html?s_z=n_C60491"/>
+    <hyperlink ref="J24" r:id="rId19" display="https://www.lcsc.com/product-detail/C105871.html?s_z=n_C105871"/>
+    <hyperlink ref="J25" r:id="rId20" display="https://www.lcsc.com/product-detail/C105875.html?s_z=n_C105875"/>
+    <hyperlink ref="J26" r:id="rId21" display="https://www.lcsc.com/product-detail/C138044.html?s_z=n_C138044"/>
+    <hyperlink ref="J27" r:id="rId22" display="https://www.lcsc.com/product-detail/C138010.html?s_z=n_C138010"/>
+    <hyperlink ref="J28" r:id="rId23" display="https://www.lcsc.com/product-detail/C105872.html?s_z=n_C105872"/>
+    <hyperlink ref="J29" r:id="rId24" display="https://www.lcsc.com/product-detail/C114762.html?s_z=n_C114762"/>
+    <hyperlink ref="J30" r:id="rId25" display="https://www.lcsc.com/product-detail/C2760981.html?s_z=n_C2760981"/>
+    <hyperlink ref="J31" r:id="rId26" display="https://www.lcsc.com/product-detail/C60490.html?s_z=n_C60490"/>
+    <hyperlink ref="J32" r:id="rId27" display="https://www.lcsc.com/product-detail/C77131.html?s_z=n_C77131"/>
+    <hyperlink ref="J33" r:id="rId28" display="https://www.lcsc.com/product-detail/C2913206.html?s_z=n_C2913206"/>
+    <hyperlink ref="J34" r:id="rId29" display="https://www.lcsc.com/product-detail/C2682616.html?s_z=n_C2682616"/>
+    <hyperlink ref="J35" r:id="rId30" display="https://www.lcsc.com/product-detail/C99269.html?s_z=n_C99269"/>
+    <hyperlink ref="J36" r:id="rId31" display="https://www.lcsc.com/product-detail/C2869734.html?s_z=n_C2869734"/>
+    <hyperlink ref="N36" r:id="rId32" display="https://www.mouser.com/ProductDetail/Texas-Instruments/LM66100DCKT?qs=vLWxofP3U2zoiBCtDTudjw%3D%3D"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>